<commit_message>
My first python project with decolabs
</commit_message>
<xml_diff>
--- a/Excel/Practice/Day1-Lookup-Formula-Practice.xlsx
+++ b/Excel/Practice/Day1-Lookup-Formula-Practice.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adebayo Olumide\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adebayo Olumide\Desktop\My-DataAnalyst-Portfolio\Excel\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC6F2958-C1ED-46E4-9A4E-264D5B8FC9E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB744DEA-CE59-448C-B9E1-26F457F60AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sales Data'!$A$3:$J$33</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="13" t="str">
-        <f>VLOOKUP(D4,'Reference Tables'!A4:B14,2,)</f>
+        <f>VLOOKUP(D4,'Reference Tables'!A5:D14,2,FALSE)</f>
         <v>Displays</v>
       </c>
       <c r="G4" s="6" t="s">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="13">
-        <f>INDEX('Reference Tables'!C4:C14,MATCH(Exercises!D5,'Reference Tables'!A4:A14,0))</f>
+        <f>INDEX('Reference Tables'!C5:C14,MATCH(Exercises!D5,'Reference Tables'!A5:A14,0))</f>
         <v>42000</v>
       </c>
       <c r="G5" s="6" t="s">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="E6" s="12"/>
       <c r="F6" s="13" t="str">
-        <f>_xlfn.XLOOKUP(D6,'Reference Tables'!F4:F10,'Reference Tables'!G4:G10)</f>
+        <f>_xlfn.XLOOKUP(D6,'Reference Tables'!F5:F10,'Reference Tables'!G5:G10,"Not Found",0)</f>
         <v>Lagos</v>
       </c>
       <c r="G6" s="6" t="s">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="13" t="str">
-        <f>_xlfn.XLOOKUP(D7,'Reference Tables'!A4:A14,'Reference Tables'!B4:B14,"Not Found")</f>
+        <f>_xlfn.XLOOKUP(Exercises!D7,'Reference Tables'!A5:A14,'Reference Tables'!B5:B14,"Not Found",0)</f>
         <v>Not Found</v>
       </c>
       <c r="G7" s="6" t="s">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="13" t="str">
-        <f>IFERROR(VLOOKUP(D8,'Reference Tables'!F4:H10,3,FALSE),"Check Name")</f>
+        <f>IFERROR(VLOOKUP(D8,'Reference Tables'!F5:I10,3,FALSE),"Check Name")</f>
         <v>Check Name</v>
       </c>
       <c r="G8" s="6" t="s">
@@ -2638,7 +2638,7 @@
         <v>18</v>
       </c>
       <c r="F9" s="13">
-        <f>INDEX('Sales Data'!A3:J33,MATCH(Exercises!D9,'Sales Data'!A3:A33,0),MATCH(Exercises!E9,'Sales Data'!A3:J3,0))</f>
+        <f>INDEX('Sales Data'!A4:J33,MATCH(Exercises!D9,'Sales Data'!A4:A33,0),MATCH(Exercises!E9,'Sales Data'!A3:J3,0))</f>
         <v>154000</v>
       </c>
       <c r="G9" s="6" t="s">

</xml_diff>